<commit_message>
docs: record Feishu webhook batch evidence
</commit_message>
<xml_diff>
--- a/docs/evaluation/shopops-operation-report-sample.xlsx
+++ b/docs/evaluation/shopops-operation-report-sample.xlsx
@@ -100,7 +100,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>XLSX-20260723231649512</t>
+          <t>XLSX-20260724011620095</t>
         </is>
       </c>
     </row>
@@ -112,7 +112,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-23T23:16:49.524705600</t>
+          <t>2026-07-24T01:16:20.116654200</t>
         </is>
       </c>
     </row>

</xml_diff>